<commit_message>
Fix formula corruption and bad output path in build_scenario_b.py
Seven 'Premissa / Fonte' cells started with "= " (e.g. "= custo final
acima - TP."), so openpyxl/Excel wrote them as formulas instead of
plain text - same root cause fixed earlier in the P&L tabs (commit
8273c75). This corrupted sheet1.xml and would trigger Excel's
'unreadable content' repair prompt. Reworded the seven notes without a
leading '=' (kept the meaning). Also fixed OUT pointing at a
nonexistent 'Proposal/' subfolder, which made the script fail to save
outside the exact environment it was first run in. Rebuilt and
verified zero text-as-formula entries remain; scenario totals
unchanged (Cenario A R$7,170,137.28 / Cenario B R$6,728,109.30,
saving R$442,027.97 / 6.16%).
</commit_message>
<xml_diff>
--- a/Pathfinder_Cost_Summary_PT_Cenario_B_RegimeEspecial.xlsx
+++ b/Pathfinder_Cost_Summary_PT_Cenario_B_RegimeEspecial.xlsx
@@ -1371,9 +1371,10 @@
         <f>C50/$C$6</f>
         <v/>
       </c>
-      <c r="E50" s="8">
-        <f> custo final acima - TP.</f>
-        <v/>
+      <c r="E50" s="8" t="inlineStr">
+        <is>
+          <t>Custo final acima menos TP.</t>
+        </is>
       </c>
     </row>
     <row r="51">
@@ -1490,9 +1491,10 @@
         <f>C56/$C$6</f>
         <v/>
       </c>
-      <c r="E56" s="19">
-        <f> ICMS acumulado + IPI.</f>
-        <v/>
+      <c r="E56" s="19" t="inlineStr">
+        <is>
+          <t>ICMS acumulado mais IPI.</t>
+        </is>
       </c>
     </row>
     <row r="58">
@@ -1561,9 +1563,10 @@
         <f>C61/$C$6</f>
         <v/>
       </c>
-      <c r="E61" s="8">
-        <f> custo acima - TP.</f>
-        <v/>
+      <c r="E61" s="8" t="inlineStr">
+        <is>
+          <t>Custo acima menos TP.</t>
+        </is>
       </c>
     </row>
     <row r="62">
@@ -1680,9 +1683,10 @@
         <f>C67/$C$6</f>
         <v/>
       </c>
-      <c r="E67" s="8">
-        <f> ICMS + IPI acima.</f>
-        <v/>
+      <c r="E67" s="8" t="inlineStr">
+        <is>
+          <t>ICMS mais IPI acima.</t>
+        </is>
       </c>
     </row>
     <row r="69">
@@ -1786,9 +1790,10 @@
         <f>C74/$C$6</f>
         <v/>
       </c>
-      <c r="E74" s="8">
-        <f> ICMS regime especial + IPI regime especial.</f>
-        <v/>
+      <c r="E74" s="8" t="inlineStr">
+        <is>
+          <t>ICMS regime especial mais IPI regime especial.</t>
+        </is>
       </c>
     </row>
     <row r="76">
@@ -1872,9 +1877,10 @@
         <f>C80/$C$6</f>
         <v/>
       </c>
-      <c r="E80" s="8">
-        <f> PIS/COFINS acumulado + ISS.</f>
-        <v/>
+      <c r="E80" s="8" t="inlineStr">
+        <is>
+          <t>PIS/COFINS acumulado mais ISS.</t>
+        </is>
       </c>
     </row>
     <row r="82">
@@ -1891,9 +1897,10 @@
         <f>C82/$C$6</f>
         <v/>
       </c>
-      <c r="E82" s="14">
-        <f> parte nao-Supermetal + parte material Supermetal (regime especial) + parte servico Supermetal (ISS).</f>
-        <v/>
+      <c r="E82" s="14" t="inlineStr">
+        <is>
+          <t>Parte nao-Supermetal mais parte material Supermetal (regime especial) mais parte servico Supermetal (ISS).</t>
+        </is>
       </c>
     </row>
     <row r="84">
@@ -1959,9 +1966,10 @@
         <v/>
       </c>
       <c r="D87" s="7" t="n"/>
-      <c r="E87" s="8">
-        <f> diferenca / preco final Cenario A.</f>
-        <v/>
+      <c r="E87" s="8" t="inlineStr">
+        <is>
+          <t>Diferenca dividida pelo preco final do Cenario A.</t>
+        </is>
       </c>
     </row>
     <row r="89" ht="40" customHeight="1">

</xml_diff>

<commit_message>
Link Scenario B to the P&L tab live, add US reference gap check
- build_scenario_b.py now reads FX/TDM/PIS-COFINS/raw costs/TP/freight/II/
  Supermetal directly from Pathfinder_Cost_Summary_PT.xlsx's P&L sheet at
  generation time instead of hardcoded literals, so the two files can
  never silently drift apart the way the No_TP_Return exploration did.
- New section 6 in the Cenario B sheet: gap of both scenarios' Final
  Client Price (USD) against the same US$900k domestic reference used
  in the Simulacao tab and the local-taxes slide, with a Fonte note
  making clear that reference is a market input (not a US cost-build
  file) while the Brazilian side reuses the full cost+freight+tax chain
  already computed in sections 3-4 of this sheet.
- Verified: zero text-as-formula corruption; Cenario A US$1,405,909.27,
  Cenario B US$1,319,237.12, matching the independently recomputed values.
</commit_message>
<xml_diff>
--- a/Pathfinder_Cost_Summary_PT_Cenario_B_RegimeEspecial.xlsx
+++ b/Pathfinder_Cost_Summary_PT_Cenario_B_RegimeEspecial.xlsx
@@ -592,7 +592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:E90"/>
+  <dimension ref="B1:E96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1263,7 +1263,7 @@
       </c>
       <c r="E43" s="8" t="inlineStr">
         <is>
-          <t>Copiado da celula B13.</t>
+          <t>Copiado da celula B13 (ao vivo).</t>
         </is>
       </c>
     </row>
@@ -1282,7 +1282,7 @@
       </c>
       <c r="E44" s="8" t="inlineStr">
         <is>
-          <t>Copiado da celula B14.</t>
+          <t>Copiado da celula B14 (ao vivo).</t>
         </is>
       </c>
     </row>
@@ -1301,7 +1301,7 @@
       </c>
       <c r="E45" s="8" t="inlineStr">
         <is>
-          <t>Copiado da celula B15.</t>
+          <t>Copiado da celula B15 (ao vivo).</t>
         </is>
       </c>
     </row>
@@ -1972,18 +1972,101 @@
         </is>
       </c>
     </row>
-    <row r="89" ht="40" customHeight="1">
-      <c r="B89" s="26" t="inlineStr">
+    <row r="89">
+      <c r="B89" s="3" t="inlineStr">
+        <is>
+          <t>6) CHECAGEM vs. REFERENCIA DOMESTICA EUA (mesma base da aba Simulacao)</t>
+        </is>
+      </c>
+      <c r="C89" s="4" t="n"/>
+      <c r="D89" s="4" t="n"/>
+      <c r="E89" s="4" t="n"/>
+    </row>
+    <row r="90">
+      <c r="B90" s="5" t="inlineStr">
+        <is>
+          <t>Descricao</t>
+        </is>
+      </c>
+      <c r="C90" s="5" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D90" s="5" t="inlineStr">
+        <is>
+          <t>US$</t>
+        </is>
+      </c>
+      <c r="E90" s="5" t="inlineStr">
+        <is>
+          <t>Premissa / Fonte (para o time de tax)</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="B91" s="6" t="inlineStr">
+        <is>
+          <t>Preco de referencia domestico EUA (US$, input)</t>
+        </is>
+      </c>
+      <c r="C91" s="7" t="n"/>
+      <c r="D91" s="24" t="n">
+        <v>900000</v>
+      </c>
+      <c r="E91" s="8" t="inlineStr">
+        <is>
+          <t>Mesmo valor de referencia usado na aba 'Simulacao' do Pathfinder_Cost_Summary_PT.xlsx e no slide MRS_Pathfinder_Simulation_Local_Taxes_Bilingual.pptx (preco informado por Matheus para a venda domestica do Pathfinder nos EUA). Nao vem de um arquivo de custo americano - e um dado de mercado, nao um calculo. O lado brasileiro de comparacao abaixo, sim, usa a cadeia completa de custo+frete+imposto ja calculada nas secoes 3 e 4 desta aba.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="B92" s="6" t="inlineStr">
+        <is>
+          <t>Preco Final ao Cliente - Cenario A vs. referencia EUA (US$)</t>
+        </is>
+      </c>
+      <c r="C92" s="7" t="n"/>
+      <c r="D92" s="7">
+        <f>D56-D91</f>
+        <v/>
+      </c>
+      <c r="E92" s="8" t="inlineStr">
+        <is>
+          <t>Cenario A (secao 3) em USD, menos a referencia EUA acima.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="B93" s="21" t="inlineStr">
+        <is>
+          <t>Preco Final ao Cliente - Cenario B vs. referencia EUA (US$)</t>
+        </is>
+      </c>
+      <c r="C93" s="22" t="n"/>
+      <c r="D93" s="22">
+        <f>D82-D91</f>
+        <v/>
+      </c>
+      <c r="E93" s="14" t="inlineStr">
+        <is>
+          <t>Cenario B (secao 4) em USD, menos a referencia EUA acima.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="40" customHeight="1">
+      <c r="B95" s="26" t="inlineStr">
         <is>
           <t>IMPORTANTE: os valores de ICMS Regime Especial (1,5%), IPI (0%) e ISS (5% placeholder) precisam de confirmacao formal do time de tax/juridico antes de qualquer uso comercial ou contratual. Este arquivo existe para orientar essa conversa, nao para ser usado como preco final.</t>
         </is>
       </c>
     </row>
-    <row r="90"/>
+    <row r="96"/>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="13">
     <mergeCell ref="B84:E84"/>
     <mergeCell ref="B1:E1"/>
+    <mergeCell ref="B95:E96"/>
     <mergeCell ref="B4:E4"/>
     <mergeCell ref="B58:E58"/>
     <mergeCell ref="B13:E13"/>
@@ -1991,8 +2074,8 @@
     <mergeCell ref="B38:E38"/>
     <mergeCell ref="B47:E47"/>
     <mergeCell ref="B2:E2"/>
+    <mergeCell ref="B95:E95"/>
     <mergeCell ref="B89:E89"/>
-    <mergeCell ref="B89:E90"/>
     <mergeCell ref="B76:E76"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>